<commit_message>
Added emd case handling
</commit_message>
<xml_diff>
--- a/hostels.xlsx
+++ b/hostels.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Svelte Learning\hostel-allotment-system\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D176B9AD-7845-44F5-8BDB-AFDF4F52E9D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA70659D-34E0-41AA-A31D-B1DE53764E7A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-93" yWindow="-93" windowWidth="19386" windowHeight="12186" xr2:uid="{31E5BBD6-E541-4916-A00A-1B4931426551}"/>
   </bookViews>
@@ -116,9 +116,8 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -463,16 +462,16 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.5">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
+      <c r="B1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
     </row>

</xml_diff>